<commit_message>
algo and feature extracted result
</commit_message>
<xml_diff>
--- a/algorithms_use.xlsx
+++ b/algorithms_use.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mmeliht/Desktop/URL-Phishing-Detection/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\URL-Phishing-Detection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCD1A8D6-AA41-CF4A-90C7-775A899BF1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F30AF91F-DAE0-4D42-85EC-C077DD393E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,6 +31,9 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -1161,11 +1164,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1454,16 +1457,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K191"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.83203125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="15.5" style="3" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" style="7" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" style="3" customWidth="1"/>
     <col min="3" max="3" width="27" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.5" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>12</v>
       </c>
@@ -1480,7 +1483,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="90" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="99.75" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>177</v>
       </c>
@@ -1497,14 +1500,14 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="23" t="s">
+    <row r="3" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="24" t="s">
         <v>178</v>
       </c>
-      <c r="B3" s="23">
+      <c r="B3" s="24">
         <v>2019</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="C3" s="24" t="s">
         <v>24</v>
       </c>
       <c r="D3" s="5" t="s">
@@ -1514,10 +1517,10 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="23"/>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="24"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
       <c r="D4" s="5" t="s">
         <v>1</v>
       </c>
@@ -1525,10 +1528,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="23"/>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="24"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
       <c r="D5" s="5" t="s">
         <v>2</v>
       </c>
@@ -1536,10 +1539,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="23"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="24"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
       <c r="D6" s="5" t="s">
         <v>3</v>
       </c>
@@ -1547,10 +1550,10 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="23"/>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="24"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
       <c r="D7" s="5" t="s">
         <v>4</v>
       </c>
@@ -1558,14 +1561,14 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="23" t="s">
+    <row r="8" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="24" t="s">
         <v>179</v>
       </c>
-      <c r="B8" s="23">
+      <c r="B8" s="24">
         <v>2023</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="24" t="s">
         <v>24</v>
       </c>
       <c r="D8" s="5" t="s">
@@ -1575,10 +1578,10 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="23"/>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="24"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
       <c r="D9" s="3" t="s">
         <v>0</v>
       </c>
@@ -1586,10 +1589,10 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
+    <row r="10" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="24"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
       <c r="D10" s="5" t="s">
         <v>28</v>
       </c>
@@ -1597,10 +1600,10 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="23"/>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="24"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
       <c r="D11" s="5" t="s">
         <v>29</v>
       </c>
@@ -1608,14 +1611,14 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="23" t="s">
+    <row r="12" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="24" t="s">
         <v>180</v>
       </c>
-      <c r="B12" s="23">
+      <c r="B12" s="24">
         <v>2022</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="C12" s="24" t="s">
         <v>24</v>
       </c>
       <c r="D12" s="5" t="s">
@@ -1625,10 +1628,10 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="23"/>
-      <c r="B13" s="23"/>
-      <c r="C13" s="23"/>
+    <row r="13" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="24"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
       <c r="D13" s="5" t="s">
         <v>35</v>
       </c>
@@ -1636,10 +1639,10 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="23"/>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
+    <row r="14" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="24"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
       <c r="D14" s="5" t="s">
         <v>36</v>
       </c>
@@ -1647,10 +1650,10 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="23"/>
-      <c r="B15" s="23"/>
-      <c r="C15" s="23"/>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="24"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
       <c r="D15" s="5" t="s">
         <v>15</v>
       </c>
@@ -1658,14 +1661,14 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="23" t="s">
+    <row r="16" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="B16" s="23">
+      <c r="B16" s="24">
         <v>2021</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C16" s="24" t="s">
         <v>24</v>
       </c>
       <c r="D16" s="5" t="s">
@@ -1675,10 +1678,10 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="23"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="24"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
       <c r="D17" s="3" t="s">
         <v>42</v>
       </c>
@@ -1686,10 +1689,10 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="23"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="24"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
       <c r="D18" s="3" t="s">
         <v>43</v>
       </c>
@@ -1697,7 +1700,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="90" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" ht="99.75" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>182</v>
       </c>
@@ -1714,11 +1717,11 @@
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="23" t="s">
+    <row r="20" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="24" t="s">
         <v>183</v>
       </c>
-      <c r="B20" s="24">
+      <c r="B20" s="23">
         <v>2023</v>
       </c>
       <c r="C20" s="25" t="s">
@@ -1731,9 +1734,9 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="26"/>
-      <c r="B21" s="24"/>
+      <c r="B21" s="23"/>
       <c r="C21" s="25"/>
       <c r="D21" s="3" t="s">
         <v>51</v>
@@ -1742,9 +1745,9 @@
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="26"/>
-      <c r="B22" s="24"/>
+      <c r="B22" s="23"/>
       <c r="C22" s="25"/>
       <c r="D22" s="3" t="s">
         <v>52</v>
@@ -1753,11 +1756,11 @@
         <v>55</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="23" t="s">
+    <row r="23" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="B23" s="24">
+      <c r="B23" s="23">
         <v>2020</v>
       </c>
       <c r="C23" s="25" t="s">
@@ -1770,9 +1773,9 @@
         <v>56</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="26"/>
-      <c r="B24" s="24"/>
+      <c r="B24" s="23"/>
       <c r="C24" s="25"/>
       <c r="D24" s="3" t="s">
         <v>22</v>
@@ -1781,14 +1784,14 @@
         <v>57</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="23" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="B25" s="24">
+      <c r="B25" s="23">
         <v>2019</v>
       </c>
-      <c r="C25" s="24" t="s">
+      <c r="C25" s="23" t="s">
         <v>58</v>
       </c>
       <c r="D25" s="3" t="s">
@@ -1798,10 +1801,10 @@
         <v>59</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="26"/>
-      <c r="B26" s="24"/>
-      <c r="C26" s="24"/>
+      <c r="B26" s="23"/>
+      <c r="C26" s="23"/>
       <c r="D26" s="3" t="s">
         <v>22</v>
       </c>
@@ -1809,7 +1812,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="105" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" ht="114" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>186</v>
       </c>
@@ -1826,7 +1829,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="120" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" ht="128.25" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>187</v>
       </c>
@@ -1843,7 +1846,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="105" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" ht="99.75" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>188</v>
       </c>
@@ -1860,7 +1863,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="135" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" ht="156.75" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>189</v>
       </c>
@@ -1877,7 +1880,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="135" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" ht="128.25" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>190</v>
       </c>
@@ -1894,14 +1897,14 @@
         <v>74</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="23" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="24" t="s">
         <v>191</v>
       </c>
-      <c r="B32" s="24">
+      <c r="B32" s="23">
         <v>2023</v>
       </c>
-      <c r="C32" s="24" t="s">
+      <c r="C32" s="23" t="s">
         <v>20</v>
       </c>
       <c r="D32" s="3" t="s">
@@ -1911,10 +1914,10 @@
         <v>76</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="26"/>
-      <c r="B33" s="24"/>
-      <c r="C33" s="24"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
       <c r="D33" s="3" t="s">
         <v>1</v>
       </c>
@@ -1922,10 +1925,10 @@
         <v>77</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="26"/>
-      <c r="B34" s="24"/>
-      <c r="C34" s="24"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
       <c r="D34" s="3" t="s">
         <v>52</v>
       </c>
@@ -1933,7 +1936,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
         <v>192</v>
       </c>
@@ -1950,14 +1953,14 @@
         <v>81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" s="23" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="24" t="s">
         <v>193</v>
       </c>
-      <c r="B36" s="24">
+      <c r="B36" s="23">
         <v>2022</v>
       </c>
-      <c r="C36" s="24" t="s">
+      <c r="C36" s="23" t="s">
         <v>82</v>
       </c>
       <c r="D36" s="3" t="s">
@@ -1967,10 +1970,10 @@
         <v>84</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="26"/>
-      <c r="B37" s="24"/>
-      <c r="C37" s="24"/>
+      <c r="B37" s="23"/>
+      <c r="C37" s="23"/>
       <c r="D37" s="3" t="s">
         <v>83</v>
       </c>
@@ -1978,10 +1981,10 @@
         <v>85</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="26"/>
-      <c r="B38" s="24"/>
-      <c r="C38" s="24"/>
+      <c r="B38" s="23"/>
+      <c r="C38" s="23"/>
       <c r="D38" s="3" t="s">
         <v>21</v>
       </c>
@@ -1989,7 +1992,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="90" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" ht="99.75" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>194</v>
       </c>
@@ -2006,14 +2009,14 @@
         <v>88</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="23" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="24" t="s">
         <v>195</v>
       </c>
-      <c r="B40" s="24">
+      <c r="B40" s="23">
         <v>2021</v>
       </c>
-      <c r="C40" s="24" t="s">
+      <c r="C40" s="23" t="s">
         <v>89</v>
       </c>
       <c r="D40" s="3" t="s">
@@ -2023,10 +2026,10 @@
         <v>86</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="26"/>
-      <c r="B41" s="24"/>
-      <c r="C41" s="24"/>
+      <c r="B41" s="23"/>
+      <c r="C41" s="23"/>
       <c r="D41" s="3" t="s">
         <v>176</v>
       </c>
@@ -2034,11 +2037,11 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="23" t="s">
+    <row r="42" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="24" t="s">
         <v>196</v>
       </c>
-      <c r="B42" s="24">
+      <c r="B42" s="23">
         <v>2020</v>
       </c>
       <c r="C42" s="25" t="s">
@@ -2051,9 +2054,9 @@
         <v>92</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="26"/>
-      <c r="B43" s="24"/>
+      <c r="B43" s="23"/>
       <c r="C43" s="25"/>
       <c r="D43" s="3" t="s">
         <v>91</v>
@@ -2062,11 +2065,11 @@
         <v>93</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="23" t="s">
+    <row r="44" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="24" t="s">
         <v>197</v>
       </c>
-      <c r="B44" s="24">
+      <c r="B44" s="23">
         <v>2020</v>
       </c>
       <c r="C44" s="25" t="s">
@@ -2079,9 +2082,9 @@
         <v>98</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="26"/>
-      <c r="B45" s="24"/>
+      <c r="B45" s="23"/>
       <c r="C45" s="25"/>
       <c r="D45" s="3" t="s">
         <v>96</v>
@@ -2090,9 +2093,9 @@
         <v>99</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="26"/>
-      <c r="B46" s="24"/>
+      <c r="B46" s="23"/>
       <c r="C46" s="25"/>
       <c r="D46" s="3" t="s">
         <v>97</v>
@@ -2101,11 +2104,11 @@
         <v>100</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="23" t="s">
+    <row r="47" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="24" t="s">
         <v>198</v>
       </c>
-      <c r="B47" s="24">
+      <c r="B47" s="23">
         <v>2022</v>
       </c>
       <c r="C47" s="25" t="s">
@@ -2118,9 +2121,9 @@
         <v>103</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="26"/>
-      <c r="B48" s="24"/>
+      <c r="B48" s="23"/>
       <c r="C48" s="25"/>
       <c r="D48" s="3" t="s">
         <v>102</v>
@@ -2129,11 +2132,11 @@
         <v>104</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="23" t="s">
+    <row r="49" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="24" t="s">
         <v>199</v>
       </c>
-      <c r="B49" s="24">
+      <c r="B49" s="23">
         <v>2017</v>
       </c>
       <c r="C49" s="25" t="s">
@@ -2146,9 +2149,9 @@
         <v>106</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="26"/>
-      <c r="B50" s="24"/>
+      <c r="B50" s="23"/>
       <c r="C50" s="25"/>
       <c r="D50" s="3" t="s">
         <v>218</v>
@@ -2157,9 +2160,9 @@
         <v>107</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="26"/>
-      <c r="B51" s="24"/>
+      <c r="B51" s="23"/>
       <c r="C51" s="25"/>
       <c r="D51" s="3" t="s">
         <v>28</v>
@@ -2168,9 +2171,9 @@
         <v>108</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="26"/>
-      <c r="B52" s="24"/>
+      <c r="B52" s="23"/>
       <c r="C52" s="25"/>
       <c r="D52" s="3" t="s">
         <v>22</v>
@@ -2179,11 +2182,11 @@
         <v>109</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="23" t="s">
+    <row r="53" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="24" t="s">
         <v>200</v>
       </c>
-      <c r="B53" s="24">
+      <c r="B53" s="23">
         <v>2022</v>
       </c>
       <c r="C53" s="25" t="s">
@@ -2196,9 +2199,9 @@
         <v>110</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="26"/>
-      <c r="B54" s="24"/>
+      <c r="B54" s="23"/>
       <c r="C54" s="25"/>
       <c r="D54" s="3" t="s">
         <v>25</v>
@@ -2207,9 +2210,9 @@
         <v>111</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="26"/>
-      <c r="B55" s="24"/>
+      <c r="B55" s="23"/>
       <c r="C55" s="25"/>
       <c r="D55" s="3" t="s">
         <v>94</v>
@@ -2218,9 +2221,9 @@
         <v>27</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="26"/>
-      <c r="B56" s="24"/>
+      <c r="B56" s="23"/>
       <c r="C56" s="25"/>
       <c r="D56" s="3" t="s">
         <v>1</v>
@@ -2229,9 +2232,9 @@
         <v>112</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="26"/>
-      <c r="B57" s="24"/>
+      <c r="B57" s="23"/>
       <c r="C57" s="25"/>
       <c r="D57" s="3" t="s">
         <v>26</v>
@@ -2240,7 +2243,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="105" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:5" ht="99.75" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
         <v>201</v>
       </c>
@@ -2257,14 +2260,14 @@
         <v>115</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A59" s="23" t="s">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="24" t="s">
         <v>202</v>
       </c>
-      <c r="B59" s="24">
+      <c r="B59" s="23">
         <v>2022</v>
       </c>
-      <c r="C59" s="24" t="s">
+      <c r="C59" s="23" t="s">
         <v>67</v>
       </c>
       <c r="D59" s="3" t="s">
@@ -2274,10 +2277,10 @@
         <v>116</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="26"/>
-      <c r="B60" s="24"/>
-      <c r="C60" s="24"/>
+      <c r="B60" s="23"/>
+      <c r="C60" s="23"/>
       <c r="D60" s="3" t="s">
         <v>25</v>
       </c>
@@ -2285,10 +2288,10 @@
         <v>117</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="26"/>
-      <c r="B61" s="24"/>
-      <c r="C61" s="24"/>
+      <c r="B61" s="23"/>
+      <c r="C61" s="23"/>
       <c r="D61" s="3" t="s">
         <v>68</v>
       </c>
@@ -2296,10 +2299,10 @@
         <v>118</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="26"/>
-      <c r="B62" s="24"/>
-      <c r="C62" s="24"/>
+      <c r="B62" s="23"/>
+      <c r="C62" s="23"/>
       <c r="D62" s="3" t="s">
         <v>69</v>
       </c>
@@ -2307,7 +2310,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="120" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:5" ht="114" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
         <v>203</v>
       </c>
@@ -2324,7 +2327,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="150" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:5" ht="142.5" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
         <v>204</v>
       </c>
@@ -2341,7 +2344,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="65" spans="1:5" ht="135" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:5" ht="128.25" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
         <v>205</v>
       </c>
@@ -2358,11 +2361,11 @@
         <v>126</v>
       </c>
     </row>
-    <row r="66" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="23" t="s">
+    <row r="66" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="24" t="s">
         <v>206</v>
       </c>
-      <c r="B66" s="24">
+      <c r="B66" s="23">
         <v>2012</v>
       </c>
       <c r="C66" s="25" t="s">
@@ -2375,9 +2378,9 @@
         <v>129</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="26"/>
-      <c r="B67" s="24"/>
+      <c r="B67" s="23"/>
       <c r="C67" s="25"/>
       <c r="D67" s="3" t="s">
         <v>128</v>
@@ -2386,11 +2389,11 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="68" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="23" t="s">
+    <row r="68" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="24" t="s">
         <v>207</v>
       </c>
-      <c r="B68" s="24">
+      <c r="B68" s="23">
         <v>2022</v>
       </c>
       <c r="C68" s="25" t="s">
@@ -2403,9 +2406,9 @@
         <v>130</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="26"/>
-      <c r="B69" s="24"/>
+      <c r="B69" s="23"/>
       <c r="C69" s="25"/>
       <c r="D69" s="3" t="s">
         <v>113</v>
@@ -2414,7 +2417,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="70" spans="1:5" ht="120" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:5" ht="128.25" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
         <v>208</v>
       </c>
@@ -2431,14 +2434,14 @@
         <v>134</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A71" s="23" t="s">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="24" t="s">
         <v>209</v>
       </c>
-      <c r="B71" s="24">
+      <c r="B71" s="23">
         <v>2020</v>
       </c>
-      <c r="C71" s="24" t="s">
+      <c r="C71" s="23" t="s">
         <v>73</v>
       </c>
       <c r="D71" s="3" t="s">
@@ -2448,10 +2451,10 @@
         <v>135</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="26"/>
-      <c r="B72" s="24"/>
-      <c r="C72" s="24"/>
+      <c r="B72" s="23"/>
+      <c r="C72" s="23"/>
       <c r="D72" s="3" t="s">
         <v>141</v>
       </c>
@@ -2459,10 +2462,10 @@
         <v>136</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="26"/>
-      <c r="B73" s="24"/>
-      <c r="C73" s="24"/>
+      <c r="B73" s="23"/>
+      <c r="C73" s="23"/>
       <c r="D73" s="3" t="s">
         <v>142</v>
       </c>
@@ -2470,10 +2473,10 @@
         <v>137</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="26"/>
-      <c r="B74" s="24"/>
-      <c r="C74" s="24"/>
+      <c r="B74" s="23"/>
+      <c r="C74" s="23"/>
       <c r="D74" s="3" t="s">
         <v>139</v>
       </c>
@@ -2481,11 +2484,11 @@
         <v>217</v>
       </c>
     </row>
-    <row r="75" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="23" t="s">
+    <row r="75" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="24" t="s">
         <v>210</v>
       </c>
-      <c r="B75" s="24">
+      <c r="B75" s="23">
         <v>2021</v>
       </c>
       <c r="C75" s="25" t="s">
@@ -2498,9 +2501,9 @@
         <v>144</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="26"/>
-      <c r="B76" s="24"/>
+      <c r="B76" s="23"/>
       <c r="C76" s="25"/>
       <c r="D76" s="3" t="s">
         <v>143</v>
@@ -2509,9 +2512,9 @@
         <v>145</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="26"/>
-      <c r="B77" s="24"/>
+      <c r="B77" s="23"/>
       <c r="C77" s="25"/>
       <c r="D77" s="3" t="s">
         <v>147</v>
@@ -2520,9 +2523,9 @@
         <v>146</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="26"/>
-      <c r="B78" s="24"/>
+      <c r="B78" s="23"/>
       <c r="C78" s="25"/>
       <c r="D78" s="3" t="s">
         <v>148</v>
@@ -2531,7 +2534,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="79" spans="1:5" ht="150" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:5" ht="142.5" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
         <v>211</v>
       </c>
@@ -2548,11 +2551,11 @@
         <v>151</v>
       </c>
     </row>
-    <row r="80" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="23" t="s">
+    <row r="80" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="B80" s="24">
+      <c r="B80" s="23">
         <v>2018</v>
       </c>
       <c r="C80" s="25" t="s">
@@ -2565,9 +2568,9 @@
         <v>155</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="26"/>
-      <c r="B81" s="24"/>
+      <c r="B81" s="23"/>
       <c r="C81" s="25"/>
       <c r="D81" s="3" t="s">
         <v>153</v>
@@ -2576,9 +2579,9 @@
         <v>156</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="26"/>
-      <c r="B82" s="24"/>
+      <c r="B82" s="23"/>
       <c r="C82" s="25"/>
       <c r="D82" s="3" t="s">
         <v>154</v>
@@ -2587,9 +2590,9 @@
         <v>157</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="26"/>
-      <c r="B83" s="24"/>
+      <c r="B83" s="23"/>
       <c r="C83" s="25"/>
       <c r="D83" s="3" t="s">
         <v>17</v>
@@ -2598,11 +2601,11 @@
         <v>158</v>
       </c>
     </row>
-    <row r="84" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="23" t="s">
+    <row r="84" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="B84" s="24">
+      <c r="B84" s="23">
         <v>2017</v>
       </c>
       <c r="C84" s="25" t="s">
@@ -2615,9 +2618,9 @@
         <v>162</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="26"/>
-      <c r="B85" s="24"/>
+      <c r="B85" s="23"/>
       <c r="C85" s="25"/>
       <c r="D85" s="3" t="s">
         <v>160</v>
@@ -2626,9 +2629,9 @@
         <v>163</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="26"/>
-      <c r="B86" s="24"/>
+      <c r="B86" s="23"/>
       <c r="C86" s="25"/>
       <c r="D86" s="3" t="s">
         <v>25</v>
@@ -2637,9 +2640,9 @@
         <v>164</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="26"/>
-      <c r="B87" s="24"/>
+      <c r="B87" s="23"/>
       <c r="C87" s="25"/>
       <c r="D87" s="3" t="s">
         <v>161</v>
@@ -2648,7 +2651,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="88" spans="1:5" ht="105" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:5" ht="114" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
         <v>214</v>
       </c>
@@ -2665,7 +2668,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="89" spans="1:5" ht="90" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:5" ht="114" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
         <v>215</v>
       </c>
@@ -2682,14 +2685,14 @@
         <v>171</v>
       </c>
     </row>
-    <row r="90" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="23" t="s">
+    <row r="90" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="24" t="s">
         <v>216</v>
       </c>
-      <c r="B90" s="24">
+      <c r="B90" s="23">
         <v>2020</v>
       </c>
-      <c r="C90" s="24" t="s">
+      <c r="C90" s="23" t="s">
         <v>119</v>
       </c>
       <c r="D90" s="3" t="s">
@@ -2699,10 +2702,10 @@
         <v>37</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A91" s="23"/>
-      <c r="B91" s="24"/>
-      <c r="C91" s="24"/>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="24"/>
+      <c r="B91" s="23"/>
+      <c r="C91" s="23"/>
       <c r="D91" s="3" t="s">
         <v>25</v>
       </c>
@@ -2710,10 +2713,10 @@
         <v>173</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A92" s="23"/>
-      <c r="B92" s="24"/>
-      <c r="C92" s="24"/>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="24"/>
+      <c r="B92" s="23"/>
+      <c r="C92" s="23"/>
       <c r="D92" s="3" t="s">
         <v>34</v>
       </c>
@@ -2721,10 +2724,10 @@
         <v>174</v>
       </c>
     </row>
-    <row r="93" spans="1:5" ht="19" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="23"/>
-      <c r="B93" s="24"/>
-      <c r="C93" s="24"/>
+    <row r="93" spans="1:5" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A93" s="24"/>
+      <c r="B93" s="23"/>
+      <c r="C93" s="23"/>
       <c r="D93" s="3" t="s">
         <v>172</v>
       </c>
@@ -2732,14 +2735,14 @@
         <v>175</v>
       </c>
     </row>
-    <row r="94" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="23" t="s">
+    <row r="94" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="24" t="s">
         <v>224</v>
       </c>
-      <c r="B94" s="24">
+      <c r="B94" s="23">
         <v>2024</v>
       </c>
-      <c r="C94" s="24" t="s">
+      <c r="C94" s="23" t="s">
         <v>223</v>
       </c>
       <c r="D94" s="3" t="s">
@@ -2749,10 +2752,10 @@
         <v>221</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A95" s="23"/>
-      <c r="B95" s="24"/>
-      <c r="C95" s="24"/>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" s="24"/>
+      <c r="B95" s="23"/>
+      <c r="C95" s="23"/>
       <c r="D95" s="3" t="s">
         <v>219</v>
       </c>
@@ -2760,10 +2763,10 @@
         <v>220</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A96" s="23"/>
-      <c r="B96" s="24"/>
-      <c r="C96" s="24"/>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="24"/>
+      <c r="B96" s="23"/>
+      <c r="C96" s="23"/>
       <c r="D96" s="3" t="s">
         <v>4</v>
       </c>
@@ -2771,11 +2774,11 @@
         <v>222</v>
       </c>
     </row>
-    <row r="97" spans="1:5" ht="19" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="23" t="s">
+    <row r="97" spans="1:5" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="24" t="s">
         <v>230</v>
       </c>
-      <c r="B97" s="24">
+      <c r="B97" s="23">
         <v>2024</v>
       </c>
       <c r="C97" s="25" t="s">
@@ -2788,10 +2791,10 @@
         <v>226</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A98" s="23"/>
-      <c r="B98" s="24"/>
-      <c r="C98" s="24"/>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" s="24"/>
+      <c r="B98" s="23"/>
+      <c r="C98" s="23"/>
       <c r="D98" s="3" t="s">
         <v>4</v>
       </c>
@@ -2799,10 +2802,10 @@
         <v>227</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A99" s="23"/>
-      <c r="B99" s="24"/>
-      <c r="C99" s="24"/>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" s="24"/>
+      <c r="B99" s="23"/>
+      <c r="C99" s="23"/>
       <c r="D99" s="3" t="s">
         <v>17</v>
       </c>
@@ -2810,10 +2813,10 @@
         <v>228</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A100" s="23"/>
-      <c r="B100" s="24"/>
-      <c r="C100" s="24"/>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="24"/>
+      <c r="B100" s="23"/>
+      <c r="C100" s="23"/>
       <c r="D100" s="3" t="s">
         <v>18</v>
       </c>
@@ -2821,14 +2824,14 @@
         <v>229</v>
       </c>
     </row>
-    <row r="101" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A101" s="23" t="s">
+    <row r="101" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="24" t="s">
         <v>232</v>
       </c>
-      <c r="B101" s="24">
+      <c r="B101" s="23">
         <v>2024</v>
       </c>
-      <c r="C101" s="24" t="s">
+      <c r="C101" s="23" t="s">
         <v>233</v>
       </c>
       <c r="D101" s="3" t="s">
@@ -2838,10 +2841,10 @@
         <v>236</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A102" s="23"/>
-      <c r="B102" s="24"/>
-      <c r="C102" s="24"/>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="24"/>
+      <c r="B102" s="23"/>
+      <c r="C102" s="23"/>
       <c r="D102" s="3" t="s">
         <v>176</v>
       </c>
@@ -2849,10 +2852,10 @@
         <v>237</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A103" s="23"/>
-      <c r="B103" s="24"/>
-      <c r="C103" s="24"/>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="24"/>
+      <c r="B103" s="23"/>
+      <c r="C103" s="23"/>
       <c r="D103" s="3" t="s">
         <v>17</v>
       </c>
@@ -2860,10 +2863,10 @@
         <v>238</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A104" s="23"/>
-      <c r="B104" s="24"/>
-      <c r="C104" s="24"/>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="24"/>
+      <c r="B104" s="23"/>
+      <c r="C104" s="23"/>
       <c r="D104" s="3" t="s">
         <v>52</v>
       </c>
@@ -2871,10 +2874,10 @@
         <v>239</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A105" s="23"/>
-      <c r="B105" s="24"/>
-      <c r="C105" s="24"/>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="24"/>
+      <c r="B105" s="23"/>
+      <c r="C105" s="23"/>
       <c r="D105" s="3" t="s">
         <v>4</v>
       </c>
@@ -2882,10 +2885,10 @@
         <v>240</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A106" s="23"/>
-      <c r="B106" s="24"/>
-      <c r="C106" s="24"/>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="24"/>
+      <c r="B106" s="23"/>
+      <c r="C106" s="23"/>
       <c r="D106" s="3" t="s">
         <v>225</v>
       </c>
@@ -2893,10 +2896,10 @@
         <v>241</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A107" s="23"/>
-      <c r="B107" s="24"/>
-      <c r="C107" s="24"/>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="24"/>
+      <c r="B107" s="23"/>
+      <c r="C107" s="23"/>
       <c r="D107" s="3" t="s">
         <v>234</v>
       </c>
@@ -2904,10 +2907,10 @@
         <v>242</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A108" s="23"/>
-      <c r="B108" s="24"/>
-      <c r="C108" s="24"/>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" s="24"/>
+      <c r="B108" s="23"/>
+      <c r="C108" s="23"/>
       <c r="D108" s="3" t="s">
         <v>235</v>
       </c>
@@ -2915,11 +2918,11 @@
         <v>243</v>
       </c>
     </row>
-    <row r="109" spans="1:5" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A109" s="23" t="s">
+    <row r="109" spans="1:5" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="24" t="s">
         <v>244</v>
       </c>
-      <c r="B109" s="24">
+      <c r="B109" s="23">
         <v>2024</v>
       </c>
       <c r="C109" s="25" t="s">
@@ -2932,10 +2935,10 @@
         <v>260</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A110" s="23"/>
-      <c r="B110" s="24"/>
-      <c r="C110" s="24"/>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" s="24"/>
+      <c r="B110" s="23"/>
+      <c r="C110" s="23"/>
       <c r="D110" s="3" t="s">
         <v>15</v>
       </c>
@@ -2943,10 +2946,10 @@
         <v>261</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A111" s="23"/>
-      <c r="B111" s="24"/>
-      <c r="C111" s="24"/>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A111" s="24"/>
+      <c r="B111" s="23"/>
+      <c r="C111" s="23"/>
       <c r="D111" s="3" t="s">
         <v>245</v>
       </c>
@@ -2954,14 +2957,14 @@
         <v>262</v>
       </c>
     </row>
-    <row r="112" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A112" s="23" t="s">
+    <row r="112" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="24" t="s">
         <v>250</v>
       </c>
-      <c r="B112" s="24">
+      <c r="B112" s="23">
         <v>2025</v>
       </c>
-      <c r="C112" s="24"/>
+      <c r="C112" s="23"/>
       <c r="D112" s="3" t="s">
         <v>246</v>
       </c>
@@ -2969,10 +2972,10 @@
         <v>263</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A113" s="23"/>
-      <c r="B113" s="24"/>
-      <c r="C113" s="24"/>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A113" s="24"/>
+      <c r="B113" s="23"/>
+      <c r="C113" s="23"/>
       <c r="D113" s="3" t="s">
         <v>247</v>
       </c>
@@ -2980,10 +2983,10 @@
         <v>86</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A114" s="23"/>
-      <c r="B114" s="24"/>
-      <c r="C114" s="24"/>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A114" s="24"/>
+      <c r="B114" s="23"/>
+      <c r="C114" s="23"/>
       <c r="D114" s="3" t="s">
         <v>248</v>
       </c>
@@ -2991,10 +2994,10 @@
         <v>86</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A115" s="23"/>
-      <c r="B115" s="24"/>
-      <c r="C115" s="24"/>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A115" s="24"/>
+      <c r="B115" s="23"/>
+      <c r="C115" s="23"/>
       <c r="D115" s="3" t="s">
         <v>249</v>
       </c>
@@ -3002,14 +3005,14 @@
         <v>264</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A116" s="23" t="s">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A116" s="24" t="s">
         <v>253</v>
       </c>
-      <c r="B116" s="24">
+      <c r="B116" s="23">
         <v>2025</v>
       </c>
-      <c r="C116" s="24"/>
+      <c r="C116" s="23"/>
       <c r="D116" s="3" t="s">
         <v>161</v>
       </c>
@@ -3017,10 +3020,10 @@
         <v>265</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A117" s="23"/>
-      <c r="B117" s="24"/>
-      <c r="C117" s="24"/>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A117" s="24"/>
+      <c r="B117" s="23"/>
+      <c r="C117" s="23"/>
       <c r="D117" s="3" t="s">
         <v>4</v>
       </c>
@@ -3028,10 +3031,10 @@
         <v>175</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A118" s="23"/>
-      <c r="B118" s="24"/>
-      <c r="C118" s="24"/>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A118" s="24"/>
+      <c r="B118" s="23"/>
+      <c r="C118" s="23"/>
       <c r="D118" s="3" t="s">
         <v>251</v>
       </c>
@@ -3039,10 +3042,10 @@
         <v>266</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A119" s="23"/>
-      <c r="B119" s="24"/>
-      <c r="C119" s="24"/>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A119" s="24"/>
+      <c r="B119" s="23"/>
+      <c r="C119" s="23"/>
       <c r="D119" s="3" t="s">
         <v>15</v>
       </c>
@@ -3050,10 +3053,10 @@
         <v>267</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A120" s="23"/>
-      <c r="B120" s="24"/>
-      <c r="C120" s="24"/>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A120" s="24"/>
+      <c r="B120" s="23"/>
+      <c r="C120" s="23"/>
       <c r="D120" s="3" t="s">
         <v>252</v>
       </c>
@@ -3061,10 +3064,10 @@
         <v>268</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A121" s="23"/>
-      <c r="B121" s="24"/>
-      <c r="C121" s="24"/>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A121" s="24"/>
+      <c r="B121" s="23"/>
+      <c r="C121" s="23"/>
       <c r="D121" s="3" t="s">
         <v>176</v>
       </c>
@@ -3072,14 +3075,14 @@
         <v>267</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A122" s="23" t="s">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A122" s="24" t="s">
         <v>271</v>
       </c>
-      <c r="B122" s="24">
+      <c r="B122" s="23">
         <v>2025</v>
       </c>
-      <c r="C122" s="24"/>
+      <c r="C122" s="23"/>
       <c r="D122" s="3" t="s">
         <v>254</v>
       </c>
@@ -3087,10 +3090,10 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A123" s="23"/>
-      <c r="B123" s="24"/>
-      <c r="C123" s="24"/>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A123" s="24"/>
+      <c r="B123" s="23"/>
+      <c r="C123" s="23"/>
       <c r="D123" s="3" t="s">
         <v>52</v>
       </c>
@@ -3098,10 +3101,10 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A124" s="23"/>
-      <c r="B124" s="24"/>
-      <c r="C124" s="24"/>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A124" s="24"/>
+      <c r="B124" s="23"/>
+      <c r="C124" s="23"/>
       <c r="D124" s="3" t="s">
         <v>234</v>
       </c>
@@ -3109,10 +3112,10 @@
         <v>0.94</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A125" s="23"/>
-      <c r="B125" s="24"/>
-      <c r="C125" s="24"/>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A125" s="24"/>
+      <c r="B125" s="23"/>
+      <c r="C125" s="23"/>
       <c r="D125" s="3" t="s">
         <v>15</v>
       </c>
@@ -3120,10 +3123,10 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A126" s="23"/>
-      <c r="B126" s="24"/>
-      <c r="C126" s="24"/>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A126" s="24"/>
+      <c r="B126" s="23"/>
+      <c r="C126" s="23"/>
       <c r="D126" s="3" t="s">
         <v>19</v>
       </c>
@@ -3131,10 +3134,10 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A127" s="23"/>
-      <c r="B127" s="24"/>
-      <c r="C127" s="24"/>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A127" s="24"/>
+      <c r="B127" s="23"/>
+      <c r="C127" s="23"/>
       <c r="D127" s="3" t="s">
         <v>18</v>
       </c>
@@ -3142,10 +3145,10 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A128" s="23"/>
-      <c r="B128" s="24"/>
-      <c r="C128" s="24"/>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A128" s="24"/>
+      <c r="B128" s="23"/>
+      <c r="C128" s="23"/>
       <c r="D128" s="3" t="s">
         <v>255</v>
       </c>
@@ -3153,10 +3156,10 @@
         <v>269</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A129" s="23"/>
-      <c r="B129" s="24"/>
-      <c r="C129" s="24"/>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A129" s="24"/>
+      <c r="B129" s="23"/>
+      <c r="C129" s="23"/>
       <c r="D129" s="3" t="s">
         <v>256</v>
       </c>
@@ -3164,10 +3167,10 @@
         <v>0.92</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A130" s="23"/>
-      <c r="B130" s="24"/>
-      <c r="C130" s="24"/>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A130" s="24"/>
+      <c r="B130" s="23"/>
+      <c r="C130" s="23"/>
       <c r="D130" s="3" t="s">
         <v>257</v>
       </c>
@@ -3175,10 +3178,10 @@
         <v>0.81</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A131" s="23"/>
-      <c r="B131" s="24"/>
-      <c r="C131" s="24"/>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A131" s="24"/>
+      <c r="B131" s="23"/>
+      <c r="C131" s="23"/>
       <c r="D131" s="3" t="s">
         <v>258</v>
       </c>
@@ -3186,10 +3189,10 @@
         <v>270</v>
       </c>
     </row>
-    <row r="132" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A132" s="23"/>
-      <c r="B132" s="24"/>
-      <c r="C132" s="24"/>
+    <row r="132" spans="1:5" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="24"/>
+      <c r="B132" s="23"/>
+      <c r="C132" s="23"/>
       <c r="D132" s="3" t="s">
         <v>259</v>
       </c>
@@ -3197,14 +3200,14 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A133" s="23" t="s">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A133" s="24" t="s">
         <v>273</v>
       </c>
-      <c r="B133" s="24">
+      <c r="B133" s="23">
         <v>2025</v>
       </c>
-      <c r="C133" s="24"/>
+      <c r="C133" s="23"/>
       <c r="D133" s="3" t="s">
         <v>17</v>
       </c>
@@ -3212,10 +3215,10 @@
         <v>0.77</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A134" s="23"/>
-      <c r="B134" s="24"/>
-      <c r="C134" s="24"/>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A134" s="24"/>
+      <c r="B134" s="23"/>
+      <c r="C134" s="23"/>
       <c r="D134" s="3" t="s">
         <v>15</v>
       </c>
@@ -3223,10 +3226,10 @@
         <v>0.81</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A135" s="23"/>
-      <c r="B135" s="24"/>
-      <c r="C135" s="24"/>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A135" s="24"/>
+      <c r="B135" s="23"/>
+      <c r="C135" s="23"/>
       <c r="D135" s="3" t="s">
         <v>16</v>
       </c>
@@ -3234,10 +3237,10 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A136" s="23"/>
-      <c r="B136" s="24"/>
-      <c r="C136" s="24"/>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A136" s="24"/>
+      <c r="B136" s="23"/>
+      <c r="C136" s="23"/>
       <c r="D136" s="3" t="s">
         <v>272</v>
       </c>
@@ -3245,14 +3248,14 @@
         <v>0.84</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A137" s="23" t="s">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A137" s="24" t="s">
         <v>276</v>
       </c>
-      <c r="B137" s="24">
+      <c r="B137" s="23">
         <v>2026</v>
       </c>
-      <c r="C137" s="24"/>
+      <c r="C137" s="23"/>
       <c r="D137" s="3" t="s">
         <v>22</v>
       </c>
@@ -3260,10 +3263,10 @@
         <v>0.94</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A138" s="23"/>
-      <c r="B138" s="24"/>
-      <c r="C138" s="24"/>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A138" s="24"/>
+      <c r="B138" s="23"/>
+      <c r="C138" s="23"/>
       <c r="D138" s="3" t="s">
         <v>52</v>
       </c>
@@ -3271,10 +3274,10 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A139" s="23"/>
-      <c r="B139" s="24"/>
-      <c r="C139" s="24"/>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A139" s="24"/>
+      <c r="B139" s="23"/>
+      <c r="C139" s="23"/>
       <c r="D139" s="3" t="s">
         <v>4</v>
       </c>
@@ -3282,10 +3285,10 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A140" s="23"/>
-      <c r="B140" s="24"/>
-      <c r="C140" s="24"/>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A140" s="24"/>
+      <c r="B140" s="23"/>
+      <c r="C140" s="23"/>
       <c r="D140" s="3" t="s">
         <v>15</v>
       </c>
@@ -3293,10 +3296,10 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A141" s="23"/>
-      <c r="B141" s="24"/>
-      <c r="C141" s="24"/>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A141" s="24"/>
+      <c r="B141" s="23"/>
+      <c r="C141" s="23"/>
       <c r="D141" s="3" t="s">
         <v>17</v>
       </c>
@@ -3304,10 +3307,10 @@
         <v>0.94</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A142" s="23"/>
-      <c r="B142" s="24"/>
-      <c r="C142" s="24"/>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A142" s="24"/>
+      <c r="B142" s="23"/>
+      <c r="C142" s="23"/>
       <c r="D142" s="3" t="s">
         <v>274</v>
       </c>
@@ -3315,10 +3318,10 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A143" s="23"/>
-      <c r="B143" s="24"/>
-      <c r="C143" s="24"/>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A143" s="24"/>
+      <c r="B143" s="23"/>
+      <c r="C143" s="23"/>
       <c r="D143" s="3" t="s">
         <v>275</v>
       </c>
@@ -3326,150 +3329,150 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="5"/>
       <c r="E144" s="15"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="5"/>
       <c r="E145" s="15"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="5"/>
       <c r="E146" s="15"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="5"/>
       <c r="E147" s="15"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="14"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="20"/>
       <c r="B149" s="14"/>
       <c r="C149" s="22"/>
       <c r="D149" s="14"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="21"/>
       <c r="B150"/>
       <c r="C150" s="13"/>
       <c r="D150"/>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="21"/>
       <c r="B151"/>
       <c r="C151" s="13"/>
       <c r="D151"/>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="21"/>
       <c r="B152"/>
       <c r="C152" s="13"/>
       <c r="D152"/>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="21"/>
       <c r="B153"/>
       <c r="C153" s="13"/>
       <c r="D153"/>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="21"/>
       <c r="B154"/>
       <c r="C154" s="13"/>
       <c r="D154"/>
       <c r="E154" s="3"/>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="21"/>
       <c r="B155"/>
       <c r="C155" s="13"/>
       <c r="D155"/>
       <c r="E155" s="3"/>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="21"/>
       <c r="B156"/>
       <c r="C156" s="13"/>
       <c r="D156"/>
       <c r="E156" s="3"/>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="21"/>
       <c r="B157"/>
       <c r="C157" s="13"/>
       <c r="D157"/>
       <c r="E157" s="3"/>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="21"/>
       <c r="B158"/>
       <c r="C158" s="13"/>
       <c r="D158"/>
       <c r="E158" s="3"/>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="21"/>
       <c r="B159"/>
       <c r="C159" s="13"/>
       <c r="D159"/>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="3"/>
       <c r="B160"/>
       <c r="C160" s="13"/>
       <c r="D160"/>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A161" s="8"/>
       <c r="B161" s="18"/>
       <c r="C161" s="17"/>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A162" s="8"/>
       <c r="B162" s="18"/>
       <c r="C162" s="17"/>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A163" s="8"/>
       <c r="B163" s="18"/>
       <c r="C163" s="17"/>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A164" s="8"/>
       <c r="B164" s="18"/>
       <c r="C164" s="17"/>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A165" s="8"/>
       <c r="B165" s="18"/>
       <c r="C165" s="17"/>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A166" s="12"/>
       <c r="B166" s="8"/>
       <c r="C166" s="10"/>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A167" s="12"/>
       <c r="B167" s="8"/>
       <c r="C167" s="10"/>
     </row>
-    <row r="168" spans="1:11" ht="19" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:11" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A168" s="19"/>
       <c r="B168"/>
       <c r="C168" s="13"/>
       <c r="E168" s="3"/>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A169" s="3"/>
       <c r="B169"/>
       <c r="C169" s="13"/>
       <c r="E169" s="3"/>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A170" s="10"/>
       <c r="B170" s="10"/>
       <c r="C170" s="10"/>
@@ -3481,7 +3484,7 @@
       <c r="J170" s="10"/>
       <c r="K170" s="10"/>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A171" s="8"/>
       <c r="B171" s="1"/>
       <c r="C171" s="8"/>
@@ -3493,7 +3496,7 @@
       <c r="J171" s="1"/>
       <c r="K171" s="1"/>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A172" s="8"/>
       <c r="B172" s="1"/>
       <c r="C172" s="8"/>
@@ -3505,7 +3508,7 @@
       <c r="J172" s="1"/>
       <c r="K172" s="1"/>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A173" s="8"/>
       <c r="B173" s="1"/>
       <c r="C173" s="8"/>
@@ -3517,7 +3520,7 @@
       <c r="J173" s="1"/>
       <c r="K173" s="1"/>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A174" s="8"/>
       <c r="B174" s="1"/>
       <c r="C174" s="8"/>
@@ -3529,7 +3532,7 @@
       <c r="J174" s="1"/>
       <c r="K174" s="1"/>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A175" s="8"/>
       <c r="B175" s="1"/>
       <c r="C175" s="8"/>
@@ -3541,7 +3544,7 @@
       <c r="J175" s="1"/>
       <c r="K175" s="1"/>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A176" s="8"/>
       <c r="B176" s="1"/>
       <c r="C176" s="8"/>
@@ -3553,7 +3556,7 @@
       <c r="J176" s="1"/>
       <c r="K176" s="1"/>
     </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A177" s="12"/>
       <c r="B177" s="16"/>
       <c r="C177" s="12"/>
@@ -3565,95 +3568,95 @@
       <c r="J177" s="11"/>
       <c r="K177" s="11"/>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A178" s="12"/>
       <c r="B178" s="8"/>
       <c r="C178" s="10"/>
       <c r="D178" s="8"/>
     </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A179" s="12"/>
       <c r="B179" s="8"/>
       <c r="C179" s="10"/>
       <c r="D179" s="8"/>
     </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A180" s="12"/>
       <c r="B180" s="8"/>
       <c r="C180" s="10"/>
       <c r="D180" s="8"/>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A181" s="10"/>
       <c r="B181" s="10"/>
       <c r="C181" s="10"/>
       <c r="D181" s="10"/>
       <c r="E181" s="10"/>
     </row>
-    <row r="182" spans="1:11" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:11" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="8"/>
       <c r="B182" s="8"/>
       <c r="C182" s="8"/>
       <c r="D182" s="8"/>
       <c r="E182" s="8"/>
     </row>
-    <row r="183" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="8"/>
       <c r="B183" s="8"/>
       <c r="C183" s="8"/>
       <c r="D183" s="8"/>
       <c r="E183" s="8"/>
     </row>
-    <row r="184" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="8"/>
       <c r="B184" s="8"/>
       <c r="C184" s="8"/>
       <c r="D184" s="8"/>
       <c r="E184" s="8"/>
     </row>
-    <row r="185" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="8"/>
       <c r="B185" s="8"/>
       <c r="C185" s="8"/>
       <c r="D185" s="8"/>
       <c r="E185" s="8"/>
     </row>
-    <row r="186" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="8"/>
       <c r="B186" s="8"/>
       <c r="C186" s="8"/>
       <c r="D186" s="8"/>
       <c r="E186" s="8"/>
     </row>
-    <row r="187" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="8"/>
       <c r="B187" s="8"/>
       <c r="C187" s="8"/>
       <c r="D187" s="8"/>
       <c r="E187" s="8"/>
     </row>
-    <row r="188" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="8"/>
       <c r="B188" s="8"/>
       <c r="C188" s="8"/>
       <c r="D188" s="8"/>
       <c r="E188" s="8"/>
     </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A189" s="8"/>
       <c r="B189" s="8"/>
       <c r="C189" s="8"/>
       <c r="D189" s="8"/>
       <c r="E189" s="8"/>
     </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A190" s="8"/>
       <c r="B190" s="8"/>
       <c r="C190" s="8"/>
       <c r="D190" s="8"/>
       <c r="E190" s="8"/>
     </row>
-    <row r="191" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="8"/>
       <c r="B191" s="8"/>
       <c r="C191" s="8"/>
@@ -3662,39 +3665,59 @@
     </row>
   </sheetData>
   <mergeCells count="96">
-    <mergeCell ref="C90:C93"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="C80:C83"/>
-    <mergeCell ref="B80:B83"/>
-    <mergeCell ref="A80:A83"/>
-    <mergeCell ref="C84:C87"/>
-    <mergeCell ref="B84:B87"/>
-    <mergeCell ref="A84:A87"/>
-    <mergeCell ref="C71:C74"/>
-    <mergeCell ref="B71:B74"/>
-    <mergeCell ref="A71:A74"/>
-    <mergeCell ref="C75:C78"/>
-    <mergeCell ref="B75:B78"/>
-    <mergeCell ref="A75:A78"/>
-    <mergeCell ref="C66:C67"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="A66:A67"/>
-    <mergeCell ref="C68:C69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="A68:A69"/>
-    <mergeCell ref="C59:C62"/>
-    <mergeCell ref="B59:B62"/>
-    <mergeCell ref="A59:A62"/>
-    <mergeCell ref="C53:C57"/>
-    <mergeCell ref="B53:B57"/>
-    <mergeCell ref="A53:A57"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="A47:A48"/>
-    <mergeCell ref="C49:C52"/>
-    <mergeCell ref="B49:B52"/>
-    <mergeCell ref="A49:A52"/>
+    <mergeCell ref="A137:A143"/>
+    <mergeCell ref="B137:B143"/>
+    <mergeCell ref="C137:C143"/>
+    <mergeCell ref="B122:B132"/>
+    <mergeCell ref="C122:C132"/>
+    <mergeCell ref="A122:A132"/>
+    <mergeCell ref="B133:B136"/>
+    <mergeCell ref="C133:C136"/>
+    <mergeCell ref="A133:A136"/>
+    <mergeCell ref="A112:A115"/>
+    <mergeCell ref="B112:B115"/>
+    <mergeCell ref="C112:C115"/>
+    <mergeCell ref="B116:B121"/>
+    <mergeCell ref="A116:A121"/>
+    <mergeCell ref="C116:C121"/>
+    <mergeCell ref="C101:C108"/>
+    <mergeCell ref="B101:B108"/>
+    <mergeCell ref="A101:A108"/>
+    <mergeCell ref="B109:B111"/>
+    <mergeCell ref="A109:A111"/>
+    <mergeCell ref="C109:C111"/>
+    <mergeCell ref="B94:B96"/>
+    <mergeCell ref="C94:C96"/>
+    <mergeCell ref="A94:A96"/>
+    <mergeCell ref="A97:A100"/>
+    <mergeCell ref="B97:B100"/>
+    <mergeCell ref="C97:C100"/>
+    <mergeCell ref="C8:C11"/>
+    <mergeCell ref="C3:C7"/>
+    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="C12:C15"/>
+    <mergeCell ref="B12:B15"/>
+    <mergeCell ref="A12:A15"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="C20:C22"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="C36:C38"/>
+    <mergeCell ref="B36:B38"/>
     <mergeCell ref="C44:C46"/>
     <mergeCell ref="B44:B46"/>
     <mergeCell ref="A44:A46"/>
@@ -3705,59 +3728,39 @@
     <mergeCell ref="C42:C43"/>
     <mergeCell ref="B42:B43"/>
     <mergeCell ref="A42:A43"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="B32:B34"/>
-    <mergeCell ref="A32:A34"/>
-    <mergeCell ref="C36:C38"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="C20:C22"/>
-    <mergeCell ref="B20:B22"/>
-    <mergeCell ref="A20:A22"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="C12:C15"/>
-    <mergeCell ref="B12:B15"/>
-    <mergeCell ref="A12:A15"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="A16:A18"/>
-    <mergeCell ref="C8:C11"/>
-    <mergeCell ref="C3:C7"/>
-    <mergeCell ref="B3:B7"/>
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="B8:B11"/>
-    <mergeCell ref="A8:A11"/>
-    <mergeCell ref="B94:B96"/>
-    <mergeCell ref="C94:C96"/>
-    <mergeCell ref="A94:A96"/>
-    <mergeCell ref="A97:A100"/>
-    <mergeCell ref="B97:B100"/>
-    <mergeCell ref="C97:C100"/>
-    <mergeCell ref="C101:C108"/>
-    <mergeCell ref="B101:B108"/>
-    <mergeCell ref="A101:A108"/>
-    <mergeCell ref="B109:B111"/>
-    <mergeCell ref="A109:A111"/>
-    <mergeCell ref="C109:C111"/>
-    <mergeCell ref="A112:A115"/>
-    <mergeCell ref="B112:B115"/>
-    <mergeCell ref="C112:C115"/>
-    <mergeCell ref="B116:B121"/>
-    <mergeCell ref="A116:A121"/>
-    <mergeCell ref="C116:C121"/>
-    <mergeCell ref="A137:A143"/>
-    <mergeCell ref="B137:B143"/>
-    <mergeCell ref="C137:C143"/>
-    <mergeCell ref="B122:B132"/>
-    <mergeCell ref="C122:C132"/>
-    <mergeCell ref="A122:A132"/>
-    <mergeCell ref="B133:B136"/>
-    <mergeCell ref="C133:C136"/>
-    <mergeCell ref="A133:A136"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="C49:C52"/>
+    <mergeCell ref="B49:B52"/>
+    <mergeCell ref="A49:A52"/>
+    <mergeCell ref="C59:C62"/>
+    <mergeCell ref="B59:B62"/>
+    <mergeCell ref="A59:A62"/>
+    <mergeCell ref="C53:C57"/>
+    <mergeCell ref="B53:B57"/>
+    <mergeCell ref="A53:A57"/>
+    <mergeCell ref="C66:C67"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="A66:A67"/>
+    <mergeCell ref="C68:C69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="A68:A69"/>
+    <mergeCell ref="C71:C74"/>
+    <mergeCell ref="B71:B74"/>
+    <mergeCell ref="A71:A74"/>
+    <mergeCell ref="C75:C78"/>
+    <mergeCell ref="B75:B78"/>
+    <mergeCell ref="A75:A78"/>
+    <mergeCell ref="C90:C93"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="C80:C83"/>
+    <mergeCell ref="B80:B83"/>
+    <mergeCell ref="A80:A83"/>
+    <mergeCell ref="C84:C87"/>
+    <mergeCell ref="B84:B87"/>
+    <mergeCell ref="A84:A87"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3767,13 +3770,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6649BA4D-B55A-4D43-AB69-0FD5D9AD3392}">
   <dimension ref="A1:C58"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.83203125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="32.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>120</v>
       </c>
@@ -3781,7 +3784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>15</v>
       </c>
@@ -3793,7 +3796,7 @@
         <v>14.788732394366198</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>17</v>
       </c>
@@ -3805,7 +3808,7 @@
         <v>8.4507042253521121</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>22</v>
       </c>
@@ -3817,7 +3820,7 @@
         <v>8.4507042253521121</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
@@ -3829,7 +3832,7 @@
         <v>7.042253521126761</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>176</v>
       </c>
@@ -3841,7 +3844,7 @@
         <v>4.929577464788732</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>52</v>
       </c>
@@ -3853,7 +3856,7 @@
         <v>4.929577464788732</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
@@ -3865,7 +3868,7 @@
         <v>4.225352112676056</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>16</v>
       </c>
@@ -3877,7 +3880,7 @@
         <v>4.225352112676056</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>29</v>
       </c>
@@ -3889,7 +3892,7 @@
         <v>3.5211267605633805</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>19</v>
       </c>
@@ -3901,7 +3904,7 @@
         <v>2.816901408450704</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>274</v>
       </c>
@@ -3913,7 +3916,7 @@
         <v>2.112676056338028</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>71</v>
       </c>
@@ -3925,7 +3928,7 @@
         <v>2.112676056338028</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>255</v>
       </c>
@@ -3937,7 +3940,7 @@
         <v>1.408450704225352</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>140</v>
       </c>
@@ -3949,7 +3952,7 @@
         <v>0.70422535211267601</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>2</v>
       </c>
@@ -3957,7 +3960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>69</v>
       </c>
@@ -3965,7 +3968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="60" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" ht="57" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>10</v>
       </c>
@@ -3973,7 +3976,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>133</v>
       </c>
@@ -3981,7 +3984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>26</v>
       </c>
@@ -3989,7 +3992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>141</v>
       </c>
@@ -3997,7 +4000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>247</v>
       </c>
@@ -4005,7 +4008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
         <v>75</v>
       </c>
@@ -4013,7 +4016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>80</v>
       </c>
@@ -4021,7 +4024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>83</v>
       </c>
@@ -4029,7 +4032,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>154</v>
       </c>
@@ -4037,7 +4040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>275</v>
       </c>
@@ -4045,7 +4048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>48</v>
       </c>
@@ -4053,7 +4056,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>172</v>
       </c>
@@ -4061,7 +4064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>96</v>
       </c>
@@ -4069,7 +4072,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>68</v>
       </c>
@@ -4077,7 +4080,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
         <v>125</v>
       </c>
@@ -4085,7 +4088,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>148</v>
       </c>
@@ -4093,7 +4096,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
         <v>150</v>
       </c>
@@ -4101,7 +4104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>235</v>
       </c>
@@ -4109,7 +4112,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>249</v>
       </c>
@@ -4117,7 +4120,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>256</v>
       </c>
@@ -4125,7 +4128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>259</v>
       </c>
@@ -4133,7 +4136,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>21</v>
       </c>
@@ -4141,7 +4144,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>160</v>
       </c>
@@ -4149,7 +4152,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>258</v>
       </c>
@@ -4157,7 +4160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>272</v>
       </c>
@@ -4165,7 +4168,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>97</v>
       </c>
@@ -4173,7 +4176,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>139</v>
       </c>
@@ -4181,7 +4184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>62</v>
       </c>
@@ -4189,7 +4192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>105</v>
       </c>
@@ -4197,7 +4200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>167</v>
       </c>
@@ -4205,7 +4208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>245</v>
       </c>
@@ -4213,7 +4216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>43</v>
       </c>
@@ -4221,7 +4224,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
         <v>65</v>
       </c>
@@ -4229,7 +4232,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>128</v>
       </c>
@@ -4237,7 +4240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>142</v>
       </c>
@@ -4245,7 +4248,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>252</v>
       </c>
@@ -4253,7 +4256,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>257</v>
       </c>
@@ -4261,7 +4264,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>246</v>
       </c>
@@ -4269,7 +4272,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>248</v>
       </c>
@@ -4277,7 +4280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="64" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
         <v>87</v>
       </c>
@@ -4285,7 +4288,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B58" s="3">
         <f>SUM(B1:B57)</f>
         <v>142</v>

</xml_diff>